<commit_message>
create new branch and add new changes
</commit_message>
<xml_diff>
--- a/Da_23_excel task_1.xlsx
+++ b/Da_23_excel task_1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\backend\data analysis 23\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\backend\data analysis 23\git hub\da23_excel_task1\da23_excel_task1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D15CA81-DE8C-4B6E-97B8-A20FA672BD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5E6D9CB5-C288-4CB4-AFF0-D6AFFE986F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Simple IF-ELSE (Electronics)" sheetId="1" r:id="rId1"/>
@@ -196,8 +196,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,121 +520,121 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>55000</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="3" t="str">
         <f>IF(B2&gt;=50000,"can buy","can not buy")</f>
         <v>can buy</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>25000</v>
       </c>
-      <c r="C3" s="4" t="str">
+      <c r="C3" s="3" t="str">
         <f>IF(B3&gt;=20000,"can buy ","can not buy")</f>
         <v xml:space="preserve">can buy </v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>2000</v>
       </c>
-      <c r="C4" s="4" t="str">
+      <c r="C4" s="3" t="str">
         <f>IF(B4&gt;=3000,"can buy","can not buy")</f>
         <v>can not buy</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>7000</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="3" t="str">
         <f>IF(B5&gt;=5000,"can buy","can not buy")</f>
         <v>can buy</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>18000</v>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="3" t="str">
         <f>IF(B6&gt;=15000,"can buy ","can not buy")</f>
         <v xml:space="preserve">can buy </v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>40000</v>
       </c>
-      <c r="C7" s="4" t="str">
+      <c r="C7" s="3" t="str">
         <f>IF(B7&gt;=30000,"can buy","can not buy")</f>
         <v>can buy</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>3500</v>
       </c>
-      <c r="C8" s="4" t="str">
+      <c r="C8" s="3" t="str">
         <f>IF(B8&gt;=3000,"can buy","can not buy")</f>
         <v>can buy</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="3">
         <v>12000</v>
       </c>
-      <c r="C9" s="4" t="str">
+      <c r="C9" s="3" t="str">
         <f>IF(B9&gt;=10000,"can buy ","can not buy")</f>
         <v xml:space="preserve">can buy </v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>15000</v>
       </c>
-      <c r="C10" s="4" t="str">
+      <c r="C10" s="3" t="str">
         <f>IF(B10&gt;=12000,"can buy","can not buy")</f>
         <v>can buy</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="3">
         <v>800</v>
       </c>
-      <c r="C11" s="4" t="str">
+      <c r="C11" s="3" t="str">
         <f>IF(B11&gt;=700,"can buy","can not buy")</f>
         <v>can buy</v>
       </c>
@@ -666,121 +666,121 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="4">
         <v>500</v>
       </c>
-      <c r="C2" s="3" t="str">
+      <c r="C2" s="4" t="str">
         <f>IF(B2&lt;1000,"Budget",IF(B2&lt;3000,"Standard",IF(B2&lt;6000,"Premium","Luxury")))</f>
         <v>Budget</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="4">
         <v>2000</v>
       </c>
-      <c r="C3" s="3" t="str">
+      <c r="C3" s="4" t="str">
         <f>IF(B3&lt;1000,"Budget",IF(B3&lt;3000,"Standard",IF(B3&lt;6000,"Premium","Luxury")))</f>
         <v>Standard</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="4">
         <v>4500</v>
       </c>
-      <c r="C4" s="3" t="str">
-        <f t="shared" ref="C2:C11" si="0">IF(B4&lt;1000,"Budget",IF(B4&lt;3000,"Standard",IF(B4&lt;6000,"Premium","Luxury")))</f>
+      <c r="C4" s="4" t="str">
+        <f t="shared" ref="C4:C10" si="0">IF(B4&lt;1000,"Budget",IF(B4&lt;3000,"Standard",IF(B4&lt;6000,"Premium","Luxury")))</f>
         <v>Premium</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="4">
         <v>8000</v>
       </c>
-      <c r="C5" s="3" t="str">
+      <c r="C5" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Luxury</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="4">
         <v>1200</v>
       </c>
-      <c r="C6" s="3" t="str">
+      <c r="C6" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Standard</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="4">
         <v>5500</v>
       </c>
-      <c r="C7" s="3" t="str">
+      <c r="C7" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Premium</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="4">
         <v>700</v>
       </c>
-      <c r="C8" s="3" t="str">
+      <c r="C8" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Budget</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="4">
         <v>9500</v>
       </c>
-      <c r="C9" s="3" t="str">
+      <c r="C9" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Luxury</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="4">
         <v>2800</v>
       </c>
-      <c r="C10" s="3" t="str">
+      <c r="C10" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Standard</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="4">
         <v>6200</v>
       </c>
-      <c r="C11" s="3" t="str">
+      <c r="C11" s="4" t="str">
         <f>IF(B11&lt;1000,"Budget",IF(B11&lt;3000,"Standard",IF(B11&lt;6000,"Premium","Luxury")))</f>
         <v>Luxury</v>
       </c>

</xml_diff>